<commit_message>
feat(CA-all): risk vs coverage - 11 senaryo (CA7 + CA8a/b/c eklendi)
CA7 + CA8a/b/c icin coverage data'lari farkli formatlarda, load fonksiyonu dual-mod:
  - finalize xlsx (Coverage_per_Mahalle veya Coverage_Gamma sayfasi)
  - long-format xlsx (scenario/mode/mahalle/coverage/R_risk sutunlari)

CA7: 04_Coverage_Gamma sayfasindan gamma=0.0 + use_mevcut=True filtrelendi.
CA8a/b/c: results/coverage_per_mahalle.xlsx, scenario=Baseline + mode=hard.

11 senaryo:
  Orig(0.249) CA1(0.671) CA2(0.614) CA3(0.546) CA4(0.546) CA5(0.546) CA6(0.546)
  CA7a(0.671) CA8a(0.757*) CA8b(0.329) CA8c(0.704)
*CA8a en yuksek monotoniklik.

Co-Authored-By: opencode <noreply@opencode>
</commit_message>
<xml_diff>
--- a/cozum_alternatifi_comparison_all/results/mahalle_risk_vs_coverage_per_scenario.xlsx
+++ b/cozum_alternatifi_comparison_all/results/mahalle_risk_vs_coverage_per_scenario.xlsx
@@ -14,7 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CA4" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CA5" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CA6" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CA7a_g1.0" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CA8a_trunc" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CA8b_adapt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CA8c_twotier" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -946,6 +950,1434 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>mahalle</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>R_risk</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>is_critical</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>coverage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>R_x_C</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>rank_R_desc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>rank_C_desc</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>diff_R_minus_C</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ABDURRAHMANGAZI</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.938451196307324</v>
+      </c>
+      <c r="E2" t="n">
+        <v>101.3765662726027</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ADIL</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.3611580744123298</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.227937453001921</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15</v>
+      </c>
+      <c r="G3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AHMET YESEVI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.033099148714698</v>
+      </c>
+      <c r="E4" t="n">
+        <v>20.45536314455102</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AKSEMSETTIN</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5.432165806654664</v>
+      </c>
+      <c r="E5" t="n">
+        <v>48.34627567922652</v>
+      </c>
+      <c r="F5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BATTALGAZI</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.073041730511138</v>
+      </c>
+      <c r="E6" t="n">
+        <v>19.74396784140494</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FATIH</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>17</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.101387373451268</v>
+      </c>
+      <c r="E7" t="n">
+        <v>35.72358534867156</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>7</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HAMIDIYE</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.041577928196808</v>
+      </c>
+      <c r="E8" t="n">
+        <v>164.8595982520356</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HASANPASA</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.792744826006886</v>
+      </c>
+      <c r="E9" t="n">
+        <v>27.07044687270398</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11</v>
+      </c>
+      <c r="G9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MECIDIYE</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9359335793815313</v>
+      </c>
+      <c r="E10" t="n">
+        <v>14.50697048041374</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MEHMET AKIF</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>31</v>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3.015708377035739</v>
+      </c>
+      <c r="E11" t="n">
+        <v>93.48695968810792</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MIMAR SINAN</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.8700338517037132</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.393132021644481</v>
+      </c>
+      <c r="F12" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NECIP FAZIL</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1.265976290635142</v>
+      </c>
+      <c r="E13" t="n">
+        <v>22.2811827151785</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ORHANGAZI</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.926954834441297</v>
+      </c>
+      <c r="E14" t="n">
+        <v>57.07561927160529</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SALGAMLI DEVLET ORMANI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>16</v>
+      </c>
+      <c r="G15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TEFERRUC TEPE ORMANI</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>16</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TURGUT REIS</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5.130619849528103</v>
+      </c>
+      <c r="E17" t="n">
+        <v>35.40127696174392</v>
+      </c>
+      <c r="F17" t="n">
+        <v>13</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>YAVUZ SELIM</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.883670302253546</v>
+      </c>
+      <c r="E18" t="n">
+        <v>32.39912919876099</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>mahalle</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>R_risk</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>is_critical</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>coverage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>R_x_C</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>rank_R_desc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>rank_C_desc</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>diff_R_minus_C</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ABDURRAHMANGAZI</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5.199652918080341</v>
+      </c>
+      <c r="E2" t="n">
+        <v>179.3880256737718</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ADIL</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.200410309213439</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.081395051325693</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15</v>
+      </c>
+      <c r="G3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AHMET YESEVI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.655536761277722</v>
+      </c>
+      <c r="E4" t="n">
+        <v>52.5796278732989</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AKSEMSETTIN</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.644340159856248</v>
+      </c>
+      <c r="E5" t="n">
+        <v>23.53462742272061</v>
+      </c>
+      <c r="F5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" t="n">
+        <v>9</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BATTALGAZI</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.847205620844287</v>
+      </c>
+      <c r="E6" t="n">
+        <v>33.98858342353488</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FATIH</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>17</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4.594701189032707</v>
+      </c>
+      <c r="E7" t="n">
+        <v>78.10992021355602</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HAMIDIYE</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3.90991633863747</v>
+      </c>
+      <c r="E8" t="n">
+        <v>127.8542642734453</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HASANPASA</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.744896856030822</v>
+      </c>
+      <c r="E9" t="n">
+        <v>41.44794252606541</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11</v>
+      </c>
+      <c r="G9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MECIDIYE</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.243662399480908</v>
+      </c>
+      <c r="E10" t="n">
+        <v>19.27676719195407</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MEHMET AKIF</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>31</v>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>6.961949067667359</v>
+      </c>
+      <c r="E11" t="n">
+        <v>215.8204210976882</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MIMAR SINAN</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.226310440465379</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4.782610717814978</v>
+      </c>
+      <c r="F12" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NECIP FAZIL</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.215912353085886</v>
+      </c>
+      <c r="E13" t="n">
+        <v>39.0000574143116</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ORHANGAZI</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.501795981422843</v>
+      </c>
+      <c r="E14" t="n">
+        <v>68.28502163774544</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SALGAMLI DEVLET ORMANI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>16</v>
+      </c>
+      <c r="G15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TEFERRUC TEPE ORMANI</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>16</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TURGUT REIS</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.121561883896467</v>
+      </c>
+      <c r="E17" t="n">
+        <v>14.63877699888562</v>
+      </c>
+      <c r="F17" t="n">
+        <v>13</v>
+      </c>
+      <c r="G17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>YAVUZ SELIM</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4.274815486531218</v>
+      </c>
+      <c r="E18" t="n">
+        <v>73.52682636833696</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n_mahalle</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n_critical</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sum_R_x_C</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sum_coverage</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>critical_coverage_sum</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>spearman_rho_R_vs_C</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>p_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Orig</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>220.38</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12.171</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.2486587163042157</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.3715056917823776</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CA1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>17</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>935.621364672892</v>
+      </c>
+      <c r="E3" t="n">
+        <v>45.54013752371351</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20.90976466378156</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.6714285714285713</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.00612776678882011</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CA2</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>17</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>908.3411621418481</v>
+      </c>
+      <c r="E4" t="n">
+        <v>45.01588563834499</v>
+      </c>
+      <c r="F4" t="n">
+        <v>20.52378354051874</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.6142857142857142</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.01483395540597696</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CA3</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1142.555479165727</v>
+      </c>
+      <c r="E5" t="n">
+        <v>52.20599211589127</v>
+      </c>
+      <c r="F5" t="n">
+        <v>28.57303571549018</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.5464285714285714</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.03506666021670982</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CA4</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>17</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1201.223733496643</v>
+      </c>
+      <c r="E6" t="n">
+        <v>54.82699502782316</v>
+      </c>
+      <c r="F6" t="n">
+        <v>30.02708691265833</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.5464285714285714</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.03506666021670982</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CA5</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>17</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1142.555479165727</v>
+      </c>
+      <c r="E7" t="n">
+        <v>52.20599211589127</v>
+      </c>
+      <c r="F7" t="n">
+        <v>28.57303571549018</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.5464285714285714</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.03506666021670982</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CA6</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>17</v>
+      </c>
+      <c r="C8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1201.223733496643</v>
+      </c>
+      <c r="E8" t="n">
+        <v>54.82699502782316</v>
+      </c>
+      <c r="F8" t="n">
+        <v>30.02708691265833</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.5464285714285714</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.03506666021670982</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CA7a_g1.0</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>17</v>
+      </c>
+      <c r="C9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D9" t="n">
+        <v>935.6213646728922</v>
+      </c>
+      <c r="E9" t="n">
+        <v>45.54013752371351</v>
+      </c>
+      <c r="F9" t="n">
+        <v>38.11992221717168</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.6714285714285713</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.00612776678882011</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CA8a_trunc</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>853.5099346617372</v>
+      </c>
+      <c r="E10" t="n">
+        <v>39.23387571355843</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.7571428571428571</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.001081108194185834</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CA8b_adapt</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>17</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>677.3480112016531</v>
+      </c>
+      <c r="E11" t="n">
+        <v>35.80252316923419</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.3285714285714285</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.2318096972061597</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CA8c_twotier</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>17</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>976.3148678844553</v>
+      </c>
+      <c r="E12" t="n">
+        <v>46.3426677655231</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.7035714285714285</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.00342433708908396</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4144,245 +5576,1057 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>scenario</t>
+          <t>mahalle</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>n_mahalle</t>
+          <t>R_risk</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>n_critical</t>
+          <t>is_critical</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>sum_R_x_C</t>
+          <t>coverage</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>sum_coverage</t>
+          <t>R_x_C</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>critical_coverage_sum</t>
+          <t>rank_R_desc</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>spearman_rho_R_vs_C</t>
+          <t>rank_C_desc</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>p_value</t>
+          <t>diff_R_minus_C</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Orig</t>
+          <t>ABDURRAHMANGAZI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
+        <v>34.5</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>220.38</v>
+        <v>3.904454475601347</v>
       </c>
       <c r="E2" t="n">
-        <v>12.171</v>
+        <v>134.7036794082465</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2486587163042157</v>
+        <v>5</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3715056917823776</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CA1</t>
+          <t>ADIL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17</v>
-      </c>
-      <c r="C3" t="n">
-        <v>5</v>
+        <v>3.4</v>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>935.621364672892</v>
+        <v>1.194788063998196</v>
       </c>
       <c r="E3" t="n">
-        <v>45.54013752371351</v>
+        <v>4.062279417593866</v>
       </c>
       <c r="F3" t="n">
-        <v>20.90976466378156</v>
+        <v>15</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6714285714285713</v>
+        <v>14</v>
       </c>
       <c r="H3" t="n">
-        <v>0.00612776678882011</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CA2</t>
+          <t>AHMET YESEVI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17</v>
-      </c>
-      <c r="C4" t="n">
-        <v>5</v>
+        <v>19.8</v>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>908.3411621418481</v>
+        <v>2.560570671301512</v>
       </c>
       <c r="E4" t="n">
-        <v>45.01588563834499</v>
+        <v>50.69929929176994</v>
       </c>
       <c r="F4" t="n">
-        <v>20.52378354051874</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6142857142857142</v>
+        <v>8</v>
       </c>
       <c r="H4" t="n">
-        <v>0.01483395540597696</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CA3</t>
+          <t>AKSEMSETTIN</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17</v>
-      </c>
-      <c r="C5" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.943588561709431</v>
+      </c>
+      <c r="E5" t="n">
+        <v>26.19793819921394</v>
+      </c>
+      <c r="F5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H5" t="n">
         <v>5</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1142.555479165727</v>
-      </c>
-      <c r="E5" t="n">
-        <v>52.20599211589127</v>
-      </c>
-      <c r="F5" t="n">
-        <v>28.57303571549018</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.5464285714285714</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.03506666021670982</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CA4</t>
+          <t>BATTALGAZI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
-      </c>
-      <c r="C6" t="n">
-        <v>5</v>
+        <v>18.4</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>1201.223733496643</v>
+        <v>1.798238320516633</v>
       </c>
       <c r="E6" t="n">
-        <v>54.82699502782316</v>
+        <v>33.08758509750604</v>
       </c>
       <c r="F6" t="n">
-        <v>30.02708691265833</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5464285714285714</v>
+        <v>13</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03506666021670982</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CA5</t>
+          <t>FATIH</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>17</v>
       </c>
-      <c r="C7" t="n">
-        <v>5</v>
+      <c r="C7" t="b">
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>1142.555479165727</v>
+        <v>4.77307465623232</v>
       </c>
       <c r="E7" t="n">
-        <v>52.20599211589127</v>
+        <v>81.14226915594945</v>
       </c>
       <c r="F7" t="n">
-        <v>28.57303571549018</v>
+        <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5464285714285714</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>0.03506666021670982</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CA6</t>
+          <t>HAMIDIYE</t>
         </is>
       </c>
       <c r="B8" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="C8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.656655318957968</v>
+      </c>
+      <c r="E8" t="n">
+        <v>184.9726289299256</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HASANPASA</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.453552970388877</v>
+      </c>
+      <c r="E9" t="n">
+        <v>37.04864985287204</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11</v>
+      </c>
+      <c r="G9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MECIDIYE</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.898112802589436</v>
+      </c>
+      <c r="E10" t="n">
+        <v>29.42074844013626</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MEHMET AKIF</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>31</v>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.777341892473296</v>
+      </c>
+      <c r="E11" t="n">
+        <v>148.0975986666722</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MIMAR SINAN</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.126734215804789</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4.394263441638677</v>
+      </c>
+      <c r="F12" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NECIP FAZIL</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.278440542374081</v>
+      </c>
+      <c r="E13" t="n">
+        <v>40.10055354578383</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ORHANGAZI</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.864602030007885</v>
+      </c>
+      <c r="E14" t="n">
+        <v>75.35973958515376</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SALGAMLI DEVLET ORMANI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>16</v>
+      </c>
+      <c r="G15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TEFERRUC TEPE ORMANI</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>16</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TURGUT REIS</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.155104465029413</v>
+      </c>
+      <c r="E17" t="n">
+        <v>14.87022080870295</v>
+      </c>
+      <c r="F17" t="n">
+        <v>13</v>
+      </c>
+      <c r="G17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>YAVUZ SELIM</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C18" t="b">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4.154878536728327</v>
+      </c>
+      <c r="E18" t="n">
+        <v>71.46391083172722</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>mahalle</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>R_risk</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>is_critical</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>coverage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>R_x_C</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>rank_R_desc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>rank_C_desc</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>diff_R_minus_C</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ABDURRAHMANGAZI</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5.101894120158306</v>
+      </c>
+      <c r="E2" t="n">
+        <v>176.0153471454616</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ADIL</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8369276339441653</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.845553955410162</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15</v>
+      </c>
+      <c r="G3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AHMET YESEVI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.989353187923296</v>
+      </c>
+      <c r="E4" t="n">
+        <v>39.38919312088126</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AKSEMSETTIN</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.69355553206081</v>
+      </c>
+      <c r="E5" t="n">
+        <v>23.97264423534121</v>
+      </c>
+      <c r="F5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BATTALGAZI</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.643479667563754</v>
+      </c>
+      <c r="E6" t="n">
+        <v>30.24002588317307</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FATIH</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>17</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3.476837408681353</v>
+      </c>
+      <c r="E7" t="n">
+        <v>59.106235947583</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" t="n">
         <v>5</v>
       </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HAMIDIYE</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
       <c r="D8" t="n">
-        <v>1201.223733496643</v>
+        <v>4.096749897058965</v>
       </c>
       <c r="E8" t="n">
-        <v>54.82699502782316</v>
+        <v>133.9637216338282</v>
       </c>
       <c r="F8" t="n">
-        <v>30.02708691265833</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5464285714285714</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>0.03506666021670982</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HASANPASA</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.465315075911853</v>
+      </c>
+      <c r="E9" t="n">
+        <v>37.22625764626898</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11</v>
+      </c>
+      <c r="G9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MECIDIYE</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.533604197063208</v>
+      </c>
+      <c r="E10" t="n">
+        <v>23.77086505447972</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MEHMET AKIF</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>31</v>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5.590024461576922</v>
+      </c>
+      <c r="E11" t="n">
+        <v>173.2907583088846</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MIMAR SINAN</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.9004252117114281</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.511658325674569</v>
+      </c>
+      <c r="F12" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NECIP FAZIL</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1.52339112436096</v>
+      </c>
+      <c r="E13" t="n">
+        <v>26.8116837887529</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ORHANGAZI</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.345849957999631</v>
+      </c>
+      <c r="E14" t="n">
+        <v>65.24407418099281</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SALGAMLI DEVLET ORMANI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>16</v>
+      </c>
+      <c r="G15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TEFERRUC TEPE ORMANI</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>16</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TURGUT REIS</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.097605655412421</v>
+      </c>
+      <c r="E17" t="n">
+        <v>7.573479022345705</v>
+      </c>
+      <c r="F17" t="n">
+        <v>13</v>
+      </c>
+      <c r="G17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>YAVUZ SELIM</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.938862582131365</v>
+      </c>
+      <c r="E18" t="n">
+        <v>50.54843641265948</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>